<commit_message>
Add safety dialogs + hardware-failure messages for Shear/Manual/Fatigue/Calibration
Frontend (index.html, js/shear.js, js/manual.js, js/fatigue.js, js/main.js, styles.css):
- Fatigue: trim Waveform dropdown to Sine/Square; neutral estimated-duration default
- Shear/Manual/Fatigue: close-mid-test Confirm/Cancel warning dialogs
- Manual: dedicated Target Force info-icon tooltip in force mode
- Shear/Manual analysis: "unavailable"/parse/no-data messages (+ .analysis-unavailable)
- Manual: align mid-move actuator-disconnect message wording

Backend (run_engine.py, server.py):
- FUTEK connect-fail + mid-run disconnect detection (shear, fatigue, calibration)
- Manual force-spike message; Zaber-disconnect wording
- Calibration: "Target force not reached" + "Load cell disconnected during calibration"
- /api/connection-check surfaces FUTEK/Zaber messages

Also commits regenerated EM + Shear sample_data analysis outputs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web_preview/sample_data/260310B01S02BA/04 17 26_50.27_Shear/Shear_Analysis_Results.xlsx
+++ b/web_preview/sample_data/260310B01S02BA/04 17 26_50.27_Shear/Shear_Analysis_Results.xlsx
@@ -33,10 +33,10 @@
     <t>Analysis Date</t>
   </si>
   <si>
-    <t>260310B01S02BA</t>
-  </si>
-  <si>
-    <t>2026-06-02 15:55:16</t>
+    <t>04 17 26_50.27_Shear</t>
+  </si>
+  <si>
+    <t>2026-06-24 15:42:35</t>
   </si>
 </sst>
 </file>

</xml_diff>